<commit_message>
adjust F05 to per-question BH and add best-method-per-question tables
</commit_message>
<xml_diff>
--- a/04_Figures/F05_prediction/c_data/F05_metrics.xlsx
+++ b/04_Figures/F05_prediction/c_data/F05_metrics.xlsx
@@ -8,6 +8,8 @@
   <sheets>
     <sheet name="classification" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="continuous" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="best_classifier_per_contrast" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="best_regressor_per_outcome" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
@@ -557,7 +559,7 @@
         <v>0.127232142857143</v>
       </c>
       <c r="K3" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="4">
@@ -627,7 +629,7 @@
         <v>0.245357142857143</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="6">
@@ -662,7 +664,7 @@
         <v>0.213839285714286</v>
       </c>
       <c r="K6" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="7">
@@ -697,7 +699,7 @@
         <v>0.154196428571429</v>
       </c>
       <c r="K7" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="8">
@@ -732,7 +734,7 @@
         <v>0.424285714285714</v>
       </c>
       <c r="K8" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="9">
@@ -767,7 +769,7 @@
         <v>0.420982142857143</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="10">
@@ -802,7 +804,7 @@
         <v>0.415089285714286</v>
       </c>
       <c r="K10" t="n">
-        <v>1</v>
+        <v>0.735607675906183</v>
       </c>
     </row>
     <row r="11">
@@ -872,7 +874,7 @@
         <v>0.119375</v>
       </c>
       <c r="K12" t="n">
-        <v>1</v>
+        <v>0.828358208955225</v>
       </c>
     </row>
     <row r="13">
@@ -1082,7 +1084,7 @@
         <v>0.449196428571429</v>
       </c>
       <c r="K18" t="n">
-        <v>1</v>
+        <v>0.828358208955225</v>
       </c>
     </row>
     <row r="19">
@@ -1467,7 +1469,7 @@
         <v>0.112232142857143</v>
       </c>
       <c r="K29" t="n">
-        <v>1</v>
+        <v>0.653731343283582</v>
       </c>
     </row>
     <row r="30">
@@ -1502,7 +1504,7 @@
         <v>0.0930357142857143</v>
       </c>
       <c r="K30" t="n">
-        <v>1</v>
+        <v>0.653731343283582</v>
       </c>
     </row>
     <row r="31">
@@ -1572,7 +1574,7 @@
         <v>0.239375</v>
       </c>
       <c r="K32" t="n">
-        <v>1</v>
+        <v>0.658848614072495</v>
       </c>
     </row>
     <row r="33">
@@ -1607,7 +1609,7 @@
         <v>0.206875</v>
       </c>
       <c r="K33" t="n">
-        <v>1</v>
+        <v>0.653731343283582</v>
       </c>
     </row>
     <row r="34">
@@ -1677,7 +1679,7 @@
         <v>0.398839285714286</v>
       </c>
       <c r="K35" t="n">
-        <v>1</v>
+        <v>0.653731343283582</v>
       </c>
     </row>
     <row r="36">
@@ -1712,7 +1714,7 @@
         <v>0.403660714285714</v>
       </c>
       <c r="K36" t="n">
-        <v>1</v>
+        <v>0.653731343283582</v>
       </c>
     </row>
     <row r="37">
@@ -1747,7 +1749,7 @@
         <v>0.392232142857143</v>
       </c>
       <c r="K37" t="n">
-        <v>1</v>
+        <v>0.658848614072495</v>
       </c>
     </row>
     <row r="38">
@@ -2152,7 +2154,7 @@
         <v>-0.185814431019672</v>
       </c>
       <c r="L2" t="n">
-        <v>0.64179104477612</v>
+        <v>0.574626865671642</v>
       </c>
       <c r="M2" t="n">
         <v>-0.147959183673469</v>
@@ -2193,7 +2195,7 @@
         <v>-0.181553328750795</v>
       </c>
       <c r="L3" t="n">
-        <v>0.841248303934871</v>
+        <v>0.895522388059702</v>
       </c>
       <c r="M3" t="n">
         <v>-0.236355799281547</v>
@@ -2234,7 +2236,7 @@
         <v>-0.165290698304909</v>
       </c>
       <c r="L4" t="n">
-        <v>0.756860857005296</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M4" t="n">
         <v>-0.180533234027299</v>
@@ -2275,7 +2277,7 @@
         <v>-0.171753375203592</v>
       </c>
       <c r="L5" t="n">
-        <v>0.64179104477612</v>
+        <v>0.485074626865671</v>
       </c>
       <c r="M5" t="n">
         <v>-0.147959183673469</v>
@@ -2316,7 +2318,7 @@
         <v>-0.187540020679328</v>
       </c>
       <c r="L6" t="n">
-        <v>0.64179104477612</v>
+        <v>0.238805970149254</v>
       </c>
       <c r="M6" t="n">
         <v>-0.00836347400793302</v>
@@ -2357,7 +2359,7 @@
         <v>-0.184081302651363</v>
       </c>
       <c r="L7" t="n">
-        <v>0.756860857005296</v>
+        <v>0.764179104477612</v>
       </c>
       <c r="M7" t="n">
         <v>-0.172887983849346</v>
@@ -2398,7 +2400,7 @@
         <v>-0.238951648372741</v>
       </c>
       <c r="L8" t="n">
-        <v>0.64179104477612</v>
+        <v>0.574626865671642</v>
       </c>
       <c r="M8" t="n">
         <v>-0.162156547469972</v>
@@ -2439,7 +2441,7 @@
         <v>-0.238405227648293</v>
       </c>
       <c r="L9" t="n">
-        <v>0.64179104477612</v>
+        <v>0.82587064676617</v>
       </c>
       <c r="M9" t="n">
         <v>-0.164791316476876</v>
@@ -2480,7 +2482,7 @@
         <v>-0.234302598719559</v>
       </c>
       <c r="L10" t="n">
-        <v>0.688863375430539</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M10" t="n">
         <v>-0.17725130007471</v>
@@ -2521,7 +2523,7 @@
         <v>-0.205599637035866</v>
       </c>
       <c r="L11" t="n">
-        <v>0.64179104477612</v>
+        <v>0.485074626865671</v>
       </c>
       <c r="M11" t="n">
         <v>-0.147959183673469</v>
@@ -2562,7 +2564,7 @@
         <v>-0.259363778981775</v>
       </c>
       <c r="L12" t="n">
-        <v>0.64179104477612</v>
+        <v>0.365671641791044</v>
       </c>
       <c r="M12" t="n">
         <v>-0.147959183673469</v>
@@ -2603,7 +2605,7 @@
         <v>-0.254757665828641</v>
       </c>
       <c r="L13" t="n">
-        <v>0.64179104477612</v>
+        <v>0.298507462686567</v>
       </c>
       <c r="M13" t="n">
         <v>0.0997227611993026</v>
@@ -2644,7 +2646,7 @@
         <v>-0.3956535787942</v>
       </c>
       <c r="L14" t="n">
-        <v>0.64179104477612</v>
+        <v>0.574626865671642</v>
       </c>
       <c r="M14" t="n">
         <v>-0.147959183673469</v>
@@ -2685,7 +2687,7 @@
         <v>-0.408814569552181</v>
       </c>
       <c r="L15" t="n">
-        <v>0.64179104477612</v>
+        <v>0.82587064676617</v>
       </c>
       <c r="M15" t="n">
         <v>-0.147959183673469</v>
@@ -2726,7 +2728,7 @@
         <v>-0.431803999177738</v>
       </c>
       <c r="L16" t="n">
-        <v>0.64179104477612</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M16" t="n">
         <v>-0.14795918367347</v>
@@ -2767,7 +2769,7 @@
         <v>-0.430453960332909</v>
       </c>
       <c r="L17" t="n">
-        <v>0.64179104477612</v>
+        <v>0.485074626865671</v>
       </c>
       <c r="M17" t="n">
         <v>-0.147959183673469</v>
@@ -2808,7 +2810,7 @@
         <v>-0.413119388289703</v>
       </c>
       <c r="L18" t="n">
-        <v>0.64179104477612</v>
+        <v>0.365671641791044</v>
       </c>
       <c r="M18" t="n">
         <v>-0.147959183673469</v>
@@ -2849,7 +2851,7 @@
         <v>-0.369765381707067</v>
       </c>
       <c r="L19" t="n">
-        <v>0.844349680170576</v>
+        <v>0.800995024875622</v>
       </c>
       <c r="M19" t="n">
         <v>-0.524480670221579</v>
@@ -2890,7 +2892,7 @@
         <v>-0.715379489498421</v>
       </c>
       <c r="L20" t="n">
-        <v>0.844349680170576</v>
+        <v>0.82089552238806</v>
       </c>
       <c r="M20" t="n">
         <v>-0.6</v>
@@ -2972,7 +2974,7 @@
         <v>-0.624575277148864</v>
       </c>
       <c r="L22" t="n">
-        <v>0.64179104477612</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M22" t="n">
         <v>-0.329385394890014</v>
@@ -3013,7 +3015,7 @@
         <v>-0.598397749471713</v>
       </c>
       <c r="L23" t="n">
-        <v>0.64179104477612</v>
+        <v>0.485074626865671</v>
       </c>
       <c r="M23" t="n">
         <v>-0.185019907607819</v>
@@ -3054,7 +3056,7 @@
         <v>-0.72881175563384</v>
       </c>
       <c r="L24" t="n">
-        <v>0.64179104477612</v>
+        <v>0.208955223880597</v>
       </c>
       <c r="M24" t="n">
         <v>0.49137091378704</v>
@@ -3095,7 +3097,7 @@
         <v>-0.711545896937507</v>
       </c>
       <c r="L25" t="n">
-        <v>0.64179104477612</v>
+        <v>0.35820895522388</v>
       </c>
       <c r="M25" t="n">
         <v>-0.0326438019885298</v>
@@ -3136,7 +3138,7 @@
         <v>-0.6946794332831</v>
       </c>
       <c r="L26" t="n">
-        <v>0.64179104477612</v>
+        <v>0.574626865671642</v>
       </c>
       <c r="M26" t="n">
         <v>-0.280212992940163</v>
@@ -3177,7 +3179,7 @@
         <v>-0.656151749610675</v>
       </c>
       <c r="L27" t="n">
-        <v>0.64179104477612</v>
+        <v>0.82587064676617</v>
       </c>
       <c r="M27" t="n">
         <v>-0.346116858235286</v>
@@ -3218,7 +3220,7 @@
         <v>-0.627100735421977</v>
       </c>
       <c r="L28" t="n">
-        <v>0.756860857005296</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M28" t="n">
         <v>-0.6</v>
@@ -3259,7 +3261,7 @@
         <v>-0.646834116967302</v>
       </c>
       <c r="L29" t="n">
-        <v>0.841248303934871</v>
+        <v>0.751243781094527</v>
       </c>
       <c r="M29" t="n">
         <v>-0.6</v>
@@ -3300,7 +3302,7 @@
         <v>-0.734651872641382</v>
       </c>
       <c r="L30" t="n">
-        <v>0.64179104477612</v>
+        <v>0.378109452736318</v>
       </c>
       <c r="M30" t="n">
         <v>-0.481583909470206</v>
@@ -3341,7 +3343,7 @@
         <v>-0.776792986971178</v>
       </c>
       <c r="L31" t="n">
-        <v>0.64179104477612</v>
+        <v>0.35820895522388</v>
       </c>
       <c r="M31" t="n">
         <v>-0.202019649113667</v>
@@ -3382,7 +3384,7 @@
         <v>-0.502115277270384</v>
       </c>
       <c r="L32" t="n">
-        <v>0.729684908789387</v>
+        <v>0.656716417910448</v>
       </c>
       <c r="M32" t="n">
         <v>-0.597120044184857</v>
@@ -3423,7 +3425,7 @@
         <v>-0.591913886638224</v>
       </c>
       <c r="L33" t="n">
-        <v>0.742004264392325</v>
+        <v>0.865671641791045</v>
       </c>
       <c r="M33" t="n">
         <v>-0.6</v>
@@ -3464,7 +3466,7 @@
         <v>-0.537676247326396</v>
       </c>
       <c r="L34" t="n">
-        <v>0.64179104477612</v>
+        <v>0.651741293532338</v>
       </c>
       <c r="M34" t="n">
         <v>-0.44982904801219</v>
@@ -3505,7 +3507,7 @@
         <v>-0.509996532237627</v>
       </c>
       <c r="L35" t="n">
-        <v>0.688863375430539</v>
+        <v>0.597014925373134</v>
       </c>
       <c r="M35" t="n">
         <v>-0.439334848140856</v>
@@ -3546,7 +3548,7 @@
         <v>-0.611684444552143</v>
       </c>
       <c r="L36" t="n">
-        <v>0.64179104477612</v>
+        <v>0.378109452736318</v>
       </c>
       <c r="M36" t="n">
         <v>-0.385492840992302</v>
@@ -3587,10 +3589,292 @@
         <v>-0.635918003061019</v>
       </c>
       <c r="L37" t="n">
-        <v>0.64179104477612</v>
+        <v>0.529850746268656</v>
       </c>
       <c r="M37" t="n">
         <v>-0.352252104779965</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.678571428571428</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.18407960199005</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.828358208955225</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.464285714285714</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.432835820895522</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.678571428571429</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.134328358208955</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.653731343283582</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>15</v>
+      </c>
+      <c r="C5" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.716417910447761</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.642857142857143</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.203980099502488</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.735607675906183</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B2" t="s">
+        <v>12</v>
+      </c>
+      <c r="C2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D2" t="n">
+        <v>-0.147959183673469</v>
+      </c>
+      <c r="E2" t="n">
+        <v>0.238805970149254</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0.574626865671642</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.0997227611993026</v>
+      </c>
+      <c r="E3" t="n">
+        <v>0.0497512437810945</v>
+      </c>
+      <c r="F3" t="n">
+        <v>0.298507462686567</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" t="n">
+        <v>0.49137091378704</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0.0348258706467662</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.208955223880597</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>33</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>13</v>
+      </c>
+      <c r="D5" t="n">
+        <v>-0.147959183673469</v>
+      </c>
+      <c r="E5" t="n">
+        <v>0.328358208955224</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.82587064676617</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B6" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-0.14795918367347</v>
+      </c>
+      <c r="E6" t="n">
+        <v>0.427860696517413</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.651741293532338</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-0.147959183673469</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.318407960199005</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.485074626865671</v>
       </c>
     </row>
   </sheetData>

</xml_diff>